<commit_message>
Review workbook: readable column names
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RLjJb3Wq5Q2cbr99Sz9XTW
</commit_message>
<xml_diff>
--- a/paper/review_workbook.xlsx
+++ b/paper/review_workbook.xlsx
@@ -589,22 +589,22 @@
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>smb_uam</t>
+          <t>smb uam</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>smb_activation</t>
+          <t>smb activation</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>smb_delivery</t>
+          <t>smb delivery</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>safety_limits</t>
+          <t>safety limits</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>carb_absorption</t>
+          <t>carb absorption</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
@@ -2431,22 +2431,22 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>smb_uam</t>
+          <t>smb uam</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>smb_activation</t>
+          <t>smb activation</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>smb_delivery</t>
+          <t>smb delivery</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>safety_limits</t>
+          <t>safety limits</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>carb_absorption</t>
+          <t>carb absorption</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
@@ -10022,22 +10022,22 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>smb_uam</t>
+          <t>smb uam</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>smb_activation</t>
+          <t>smb activation</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>smb_delivery</t>
+          <t>smb delivery</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>safety_limits</t>
+          <t>safety limits</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -10047,7 +10047,7 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>carb_absorption</t>
+          <t>carb absorption</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
@@ -17841,22 +17841,22 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>smb_uam</t>
+          <t>smb uam</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>smb_activation</t>
+          <t>smb activation</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>smb_delivery</t>
+          <t>smb delivery</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>safety_limits</t>
+          <t>safety limits</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -17866,7 +17866,7 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>carb_absorption</t>
+          <t>carb absorption</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
@@ -24988,22 +24988,22 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>smb_uam</t>
+          <t>smb uam</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>smb_activation</t>
+          <t>smb activation</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>smb_delivery</t>
+          <t>smb delivery</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>safety_limits</t>
+          <t>safety limits</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -25013,7 +25013,7 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>carb_absorption</t>
+          <t>carb absorption</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
@@ -32807,22 +32807,22 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>smb_uam</t>
+          <t>smb uam</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>smb_activation</t>
+          <t>smb activation</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>smb_delivery</t>
+          <t>smb delivery</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>safety_limits</t>
+          <t>safety limits</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -32832,7 +32832,7 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>carb_absorption</t>
+          <t>carb absorption</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
@@ -40626,22 +40626,22 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>smb_uam</t>
+          <t>smb uam</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>smb_activation</t>
+          <t>smb activation</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>smb_delivery</t>
+          <t>smb delivery</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>safety_limits</t>
+          <t>safety limits</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -40651,7 +40651,7 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>carb_absorption</t>
+          <t>carb absorption</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
@@ -47213,22 +47213,22 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>smb_uam</t>
+          <t>smb uam</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>smb_activation</t>
+          <t>smb activation</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>smb_delivery</t>
+          <t>smb delivery</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>safety_limits</t>
+          <t>safety limits</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -47238,7 +47238,7 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>carb_absorption</t>
+          <t>carb absorption</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
@@ -55032,22 +55032,22 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>smb_uam</t>
+          <t>smb uam</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>smb_activation</t>
+          <t>smb activation</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>smb_delivery</t>
+          <t>smb delivery</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>safety_limits</t>
+          <t>safety limits</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -55057,7 +55057,7 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>carb_absorption</t>
+          <t>carb absorption</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
@@ -62627,22 +62627,22 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>smb_uam</t>
+          <t>smb uam</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>smb_activation</t>
+          <t>smb activation</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>smb_delivery</t>
+          <t>smb delivery</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>safety_limits</t>
+          <t>safety limits</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -62652,7 +62652,7 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>carb_absorption</t>
+          <t>carb absorption</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
@@ -64878,22 +64878,22 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>smb_uam</t>
+          <t>smb uam</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>smb_activation</t>
+          <t>smb activation</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>smb_delivery</t>
+          <t>smb delivery</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>safety_limits</t>
+          <t>safety limits</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -64903,7 +64903,7 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>carb_absorption</t>
+          <t>carb absorption</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
@@ -68025,22 +68025,22 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>smb_uam</t>
+          <t>smb uam</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>smb_activation</t>
+          <t>smb activation</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>smb_delivery</t>
+          <t>smb delivery</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>safety_limits</t>
+          <t>safety limits</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -68050,7 +68050,7 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>carb_absorption</t>
+          <t>carb absorption</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">

</xml_diff>